<commit_message>
Replace body-weight questions and options in both sets
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012At1DdBHCbmKTSWhAZPRk5
</commit_message>
<xml_diff>
--- a/sets/grade7-theme1-set1/questions.xlsx
+++ b/sets/grade7-theme1-set1/questions.xlsx
@@ -519,7 +519,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>She is tall and slim with blue eyes.</t>
+          <t>She is tall with long hair and blue eyes.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -565,7 +565,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>He is well-built.</t>
+          <t>He is tall and handsome.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -872,7 +872,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>plump</t>
+          <t>blonde</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>plump</t>
+          <t>lazy</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
@@ -1090,7 +1090,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>slim</t>
+          <t>rude</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr"/>
@@ -1213,7 +1213,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>plump</t>
+          <t>lazy</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr"/>
@@ -1233,28 +1233,28 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Which word means 'a little fat'?</t>
+          <t>Which word do we use for a sweet baby or a little kitten?</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr"/>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>plump</t>
+          <t>cute</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>well-built</t>
+          <t>lazy</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>tall</t>
+          <t>stubborn</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>slim</t>
+          <t>handsome</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr"/>
@@ -1266,7 +1266,7 @@
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>Opposite of slim.</t>
+          <t>small and sweet</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr"/>
@@ -1326,17 +1326,17 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
+          <t>old</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>handsome</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
           <t>young</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>thin</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>slim</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Vocabulary blanks instead of connectors, simple comparatives only, no beard option
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012At1DdBHCbmKTSWhAZPRk5
</commit_message>
<xml_diff>
--- a/sets/grade7-theme1-set1/questions.xlsx
+++ b/sets/grade7-theme1-set1/questions.xlsx
@@ -672,7 +672,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Look at Grandpa Kemal. What does he look like?</t>
+          <t>Look at Grandpa Kemal. He is ______. He has got a white moustache and glasses.</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -682,22 +682,22 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>He is young and he has got curly hair.</t>
+          <t>pretty</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>He is old. He has got long blonde hair.</t>
+          <t>cute</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>He is young. He has got a black beard.</t>
+          <t>young</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>He is old. He has got a white moustache and glasses.</t>
+          <t>old</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
@@ -709,7 +709,7 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Look at his face and his hair.</t>
+          <t>Look at his hair. It is gray.</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr"/>
@@ -1526,7 +1526,7 @@
       <c r="B26" s="2" t="inlineStr"/>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>tallest</t>
+          <t>more taller</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1571,22 +1571,22 @@
       <c r="B27" s="2" t="inlineStr"/>
       <c r="C27" s="2" t="inlineStr">
         <is>
+          <t>more outgoinger</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>more outgoing</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
           <t>outgoing</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>more outgoing</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr">
+      <c r="F27" s="2" t="inlineStr">
         <is>
           <t>outgoinger</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>most outgoing</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr"/>
@@ -1612,22 +1612,22 @@
       <c r="B28" s="2" t="inlineStr"/>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>best</t>
+          <t>more good</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>better</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
           <t>gooder</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>better</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>more good</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr"/>
@@ -1639,7 +1639,7 @@
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>good → ______ → best</t>
+          <t>We don't say 'gooder'.</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr"/>
@@ -1647,28 +1647,28 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Helen is beautiful ______ blue eyes and long straight hair.</t>
+          <t>Helen is beautiful with blue ______ and long straight ______.</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr"/>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>than</t>
+          <t>eyes / smile</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>has</t>
+          <t>smile / hair</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>and</t>
+          <t>hair / eyes</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>with</t>
+          <t>eyes / hair</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr"/>
@@ -1680,7 +1680,7 @@
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>a girl ______ blue eyes = a girl who has blue eyes</t>
+          <t>What can be blue? What can be long and straight?</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr"/>
@@ -1688,28 +1688,28 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>I like her ______ she isn't selfish.</t>
+          <t>I like her because she isn't ______. She always shares her things.</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr"/>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>so</t>
+          <t>fair</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>but</t>
+          <t>generous</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>because</t>
+          <t>selfish</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>than</t>
+          <t>supportive</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr"/>
@@ -1721,7 +1721,7 @@
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>This word answers the question 'Why?'</t>
+          <t>Opposite of generous.</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr"/>
@@ -1729,28 +1729,28 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>They like sharing and supporting each other. ______ they are good buddies.</t>
+          <t>Arda and Can always help each other. They are very ______. That's why they are good buddies.</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr"/>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>But</t>
+          <t>stubborn</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>That's why</t>
+          <t>supportive</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Because</t>
+          <t>selfish</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Than</t>
+          <t>rude</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr"/>
@@ -1762,7 +1762,7 @@
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>It means 'so'.</t>
+          <t>They help each other.</t>
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Picture questions ask about appearance details
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012At1DdBHCbmKTSWhAZPRk5
</commit_message>
<xml_diff>
--- a/sets/grade7-theme1-set1/questions.xlsx
+++ b/sets/grade7-theme1-set1/questions.xlsx
@@ -672,7 +672,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Look at Grandpa Kemal. He is ______. He has got a white moustache and glasses.</t>
+          <t>Grandpa Kemal is old. He has got brown ______ and he wears ______.</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -682,22 +682,22 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>pretty</t>
+          <t>glasses / eyes</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>cute</t>
+          <t>eyes / a headscarf</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>young</t>
+          <t>hair / glasses</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>old</t>
+          <t>eyes / glasses</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
@@ -709,7 +709,7 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Look at his hair. It is gray.</t>
+          <t>Look at his face.</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr"/>
@@ -852,7 +852,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Mr. Can is young and ______.</t>
+          <t>Mr. Can has got short ______ hair and brown eyes. He wears glasses.</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -862,22 +862,22 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>handsome</t>
+          <t>black</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>pretty</t>
+          <t>red</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
+          <t>gray</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
           <t>blonde</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>old</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
@@ -889,7 +889,7 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>We use 'pretty' for girls.</t>
+          <t>Look at the colour of his hair.</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr"/>
@@ -942,7 +942,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Elif wears a ______. She has got brown eyes and a nice smile.</t>
+          <t>Elif has got big brown ______ and a nice ______.</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -952,22 +952,22 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>headscarf</t>
+          <t>eyes / smile</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>cap</t>
+          <t>smile / eyes</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>moustache</t>
+          <t>hair / smile</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>beanie</t>
+          <t>eyes / moustache</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
@@ -979,7 +979,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Look at her head.</t>
+          <t>Look at her eyes and her mouth.</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>

</xml_diff>